<commit_message>
feat(telephonie): diffusion WebSocket temps reel a l'ingestion + panneau live UI
Complete la tache 11bis.4 (laissee en suspens depuis la Phase 11bis) : le
panneau "Evenements ESL en temps reel" n'existait jusqu'ici que comme mockup
Artifact valide visuellement, jamais raccorde au code reel.

- Backend : POST /events/ingest emet desormais socketio.emit("telephony_event",
  ..., room=str(tenant_id), namespace="/telephony") apres persistance -
  best-effort (une panne de diffusion WS ne fait jamais echouer l'ingestion,
  l'evenement reste persiste dans tous les cas). 2 nouveaux tests.
- Frontend : composable useTelephonySocket (connexion partagee au namespace
  /telephony, buffer borne a 200 evenements) + panneau live dans
  SettingsTelephony.vue (sous-ligne par connecteur, filtrable par
  event_type, pause/effacer, masquable), fidele au mockup valide.
- Nouvelle dependance frontend : socket.io-client.

199/199 tests backend verts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/suivi_taches_permatel.xlsx
+++ b/docs/suivi_taches_permatel.xlsx
@@ -4969,12 +4969,12 @@
       </c>
       <c r="F59" s="100" t="inlineStr">
         <is>
-          <t>POST /api/telephony/events/ingest émet vers la room du tenant après persistance en base (flux unique temps réel + historisation, cf. CDC §7).</t>
+          <t>Complété le 2026-07-27 : socketio.emit("telephony_event", event.to_dict(), room=str(event.tenant_id), namespace="/telephony") dans POST /events/ingest, best-effort (une panne de diffusion WS ne fait jamais echouer l ingestion). Panneau live cote frontend : SettingsTelephony.vue (composable useTelephonySocket), filtrable par event_type, masquable. 2 nouveaux tests backend.</t>
         </is>
       </c>
       <c r="G59" s="102" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>Complété</t>
         </is>
       </c>
       <c r="H59" s="100" t="inlineStr">
@@ -6716,27 +6716,27 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="51" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="51" t="inlineStr">
         <is>
           <t>12.7-12.9</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="51" t="inlineStr">
         <is>
           <t>Pivot Phase 12 : connecteur PBX tenant-scope (comme SMTP/IMAP) + Sync temps reel Redis + heartbeat statut</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="51" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E61" s="51" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>

</xml_diff>

<commit_message>
docs: mise a jour de la documentation Telephonie (pivot tenant-scope, panneau live, 2 correctifs prod)
README v1.7.0, PROJECT_STRUCTURE, TELEPHONIE_INTEGRATION_PLAN §8.5 et
DATABASE_SCHEMA (telephony_events + pbx_connectors/pbx_connector_domains)
mis a jour pour refleter l'etat reellement livre en production ; suivi des
taches complete pour les deux correctifs (deadlock ESL, routage WS Nginx).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/suivi_taches_permatel.xlsx
+++ b/docs/suivi_taches_permatel.xlsx
@@ -1832,7 +1832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M76"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="51" min="1" max="1"/>
@@ -5438,119 +5438,83 @@
       </c>
     </row>
     <row r="69" ht="37.5" customHeight="1" s="52">
-      <c r="A69" s="98" t="inlineStr">
-        <is>
-          <t>13.1</t>
-        </is>
-      </c>
-      <c r="B69" s="99" t="inlineStr">
-        <is>
-          <t>Phase 13</t>
-        </is>
-      </c>
-      <c r="C69" s="100" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D69" s="101" t="inlineStr">
-        <is>
-          <t>🟢 Normale</t>
-        </is>
-      </c>
-      <c r="E69" s="100" t="inlineStr">
-        <is>
-          <t>SupervisionTelephonieView.vue</t>
-        </is>
-      </c>
-      <c r="F69" s="100" t="inlineStr">
-        <is>
-          <t>Calque de SupervisionView.vue existant. Charge KPIs historisés + appels actifs.</t>
-        </is>
-      </c>
-      <c r="G69" s="102" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="H69" s="100" t="inlineStr">
-        <is>
-          <t>1j</t>
-        </is>
-      </c>
-      <c r="I69" s="100" t="inlineStr">
-        <is>
-          <t>frontend/src/views/SupervisionTelephonieView.vue (nouveau)</t>
-        </is>
-      </c>
-      <c r="J69" s="100" t="inlineStr">
-        <is>
-          <t>11.4, 11.5</t>
-        </is>
-      </c>
-      <c r="K69" s="100" t="n"/>
-      <c r="L69" s="100" t="n"/>
-      <c r="M69" s="100" t="n"/>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>12.10</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Phase 12</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Connecteur</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Fix deadlock reconnexion concurrente (ESLAdapter)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Complete le 2026-07-28 : force_reconnect()/stop() ne touchent plus _esl directement (course avec run() sur ESLProtocol.stop() sans timeout, bloquait le connecteur apres Sync). _hard_disconnect() ferme la socket directement, seule la greenlet run() y touche. 5 tests de regression.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="98" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="B70" s="99" t="inlineStr">
-        <is>
-          <t>Phase 13</t>
-        </is>
-      </c>
-      <c r="C70" s="100" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D70" s="101" t="inlineStr">
-        <is>
-          <t>🟢 Normale</t>
-        </is>
-      </c>
-      <c r="E70" s="100" t="inlineStr">
-        <is>
-          <t>Composable useTelephonySocket</t>
-        </is>
-      </c>
-      <c r="F70" s="100" t="inlineStr">
-        <is>
-          <t>Connexion WebSocket (namespace /telephony), auth JWT à la connexion, rejoint la room du tenant actif, reconnexion auto. Remplace le polling initialement envisagé (décision révisée : WebSocket retenu).</t>
-        </is>
-      </c>
-      <c r="G70" s="102" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="H70" s="100" t="inlineStr">
-        <is>
-          <t>½j</t>
-        </is>
-      </c>
-      <c r="I70" s="100" t="inlineStr">
-        <is>
-          <t>frontend/src/composables/useTelephonySocket.js (nouveau)</t>
-        </is>
-      </c>
-      <c r="J70" s="100" t="inlineStr">
-        <is>
-          <t>11.5, 11bis.2</t>
-        </is>
-      </c>
-      <c r="K70" s="100" t="n"/>
-      <c r="L70" s="100" t="n"/>
-      <c r="M70" s="100" t="n"/>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>12.11</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Phase 12</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Frontend/Nginx</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Fix routage WebSocket Socket.IO (panneau live bloque Deconnecte)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Complete le 2026-07-28 : /socket.io par defaut non proxifie par Nginx (tombait dans le fallback SPA). Deplace sous /api/socket.io (same-origin) + en-tetes Upgrade/Connection ajoutes a la location /api/. Valide de bout en bout contre une vraie stack Docker (nginx + gunicorn eventlet), pas seulement en test unitaire.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="98" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="B71" s="99" t="inlineStr">
@@ -5570,12 +5534,12 @@
       </c>
       <c r="E71" s="100" t="inlineStr">
         <is>
-          <t>Store Pinia useTelephonyStore</t>
+          <t>SupervisionTelephonieView.vue</t>
         </is>
       </c>
       <c r="F71" s="100" t="inlineStr">
         <is>
-          <t>État activeCalls/alerts. Actions addOrUpdateCall, removeCall, pushAlert.</t>
+          <t>Calque de SupervisionView.vue existant. Charge KPIs historisés + appels actifs.</t>
         </is>
       </c>
       <c r="G71" s="102" t="inlineStr">
@@ -5585,17 +5549,17 @@
       </c>
       <c r="H71" s="100" t="inlineStr">
         <is>
-          <t>½j</t>
+          <t>1j</t>
         </is>
       </c>
       <c r="I71" s="100" t="inlineStr">
         <is>
-          <t>frontend/src/store/telephony.js (nouveau)</t>
+          <t>frontend/src/views/SupervisionTelephonieView.vue (nouveau)</t>
         </is>
       </c>
       <c r="J71" s="100" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>11.4, 11.5</t>
         </is>
       </c>
       <c r="K71" s="100" t="n"/>
@@ -5605,7 +5569,7 @@
     <row r="72">
       <c r="A72" s="98" t="inlineStr">
         <is>
-          <t>13.4</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="B72" s="99" t="inlineStr">
@@ -5625,12 +5589,12 @@
       </c>
       <c r="E72" s="100" t="inlineStr">
         <is>
-          <t>TelephonyKpiCards.vue / ActiveCallsTable.vue / AgentsGrid.vue</t>
+          <t>Composable useTelephonySocket</t>
         </is>
       </c>
       <c r="F72" s="100" t="inlineStr">
         <is>
-          <t>Cartes KPI, tableau des appels actifs filtrable, grille agents avec statut courant.</t>
+          <t>Connexion WebSocket (namespace /telephony), auth JWT à la connexion, rejoint la room du tenant actif, reconnexion auto. Remplace le polling initialement envisagé (décision révisée : WebSocket retenu).</t>
         </is>
       </c>
       <c r="G72" s="102" t="inlineStr">
@@ -5640,17 +5604,17 @@
       </c>
       <c r="H72" s="100" t="inlineStr">
         <is>
-          <t>2j</t>
+          <t>½j</t>
         </is>
       </c>
       <c r="I72" s="100" t="inlineStr">
         <is>
-          <t>frontend/src/components/telephony/ (nouveau)</t>
+          <t>frontend/src/composables/useTelephonySocket.js (nouveau)</t>
         </is>
       </c>
       <c r="J72" s="100" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>11.5, 11bis.2</t>
         </is>
       </c>
       <c r="K72" s="100" t="n"/>
@@ -5660,7 +5624,7 @@
     <row r="73">
       <c r="A73" s="98" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="B73" s="99" t="inlineStr">
@@ -5675,17 +5639,17 @@
       </c>
       <c r="D73" s="101" t="inlineStr">
         <is>
-          <t>🔵 Normale</t>
+          <t>🟢 Normale</t>
         </is>
       </c>
       <c r="E73" s="100" t="inlineStr">
         <is>
-          <t>Réglages connecteurs PBX (UI)</t>
+          <t>Store Pinia useTelephonyStore</t>
         </is>
       </c>
       <c r="F73" s="100" t="inlineStr">
         <is>
-          <t>Formulaire CRUD pbx_connectors dans Réglages &gt; Intégrations, sur le modèle SettingsSmtp.vue.</t>
+          <t>État activeCalls/alerts. Actions addOrUpdateCall, removeCall, pushAlert.</t>
         </is>
       </c>
       <c r="G73" s="102" t="inlineStr">
@@ -5695,17 +5659,17 @@
       </c>
       <c r="H73" s="100" t="inlineStr">
         <is>
-          <t>1j</t>
+          <t>½j</t>
         </is>
       </c>
       <c r="I73" s="100" t="inlineStr">
         <is>
-          <t>frontend/src/components/settings/SettingsTelephony.vue (nouveau)</t>
+          <t>frontend/src/store/telephony.js (nouveau)</t>
         </is>
       </c>
       <c r="J73" s="100" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="K73" s="100" t="n"/>
@@ -5715,32 +5679,32 @@
     <row r="74">
       <c r="A74" s="98" t="inlineStr">
         <is>
-          <t>14.1</t>
+          <t>13.4</t>
         </is>
       </c>
       <c r="B74" s="99" t="inlineStr">
         <is>
-          <t>Phase 14</t>
+          <t>Phase 13</t>
         </is>
       </c>
       <c r="C74" s="100" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D74" s="101" t="inlineStr">
         <is>
-          <t>🔵 Normale</t>
+          <t>🟢 Normale</t>
         </is>
       </c>
       <c r="E74" s="100" t="inlineStr">
         <is>
-          <t>AMIAdapter (Asterisk) — ajouté au même process connecteur</t>
+          <t>TelephonyKpiCards.vue / ActiveCallsTable.vue / AgentsGrid.vue</t>
         </is>
       </c>
       <c r="F74" s="100" t="inlineStr">
         <is>
-          <t>Implémente PBXAdapter, orchestré par le même Core Connector que l'ESLAdapter (pas un second déploiement) : Dial/Hangup/QueueMember normalisés vers le même format standard.</t>
+          <t>Cartes KPI, tableau des appels actifs filtrable, grille agents avec statut courant.</t>
         </is>
       </c>
       <c r="G74" s="102" t="inlineStr">
@@ -5755,12 +5719,12 @@
       </c>
       <c r="I74" s="100" t="inlineStr">
         <is>
-          <t>telephony-connector/adapters/ami.py (nouveau)</t>
+          <t>frontend/src/components/telephony/ (nouveau)</t>
         </is>
       </c>
       <c r="J74" s="100" t="inlineStr">
         <is>
-          <t>12.2, 12.4</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="K74" s="100" t="n"/>
@@ -5770,17 +5734,17 @@
     <row r="75">
       <c r="A75" s="98" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="B75" s="99" t="inlineStr">
         <is>
-          <t>Phase 14</t>
+          <t>Phase 13</t>
         </is>
       </c>
       <c r="C75" s="100" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D75" s="101" t="inlineStr">
@@ -5790,12 +5754,12 @@
       </c>
       <c r="E75" s="100" t="inlineStr">
         <is>
-          <t>Validation architecture Adapter (non-régression ESL)</t>
+          <t>Réglages connecteurs PBX (UI)</t>
         </is>
       </c>
       <c r="F75" s="100" t="inlineStr">
         <is>
-          <t>Vérifier qu'aucun changement API/frontend n'est requis pour supporter Asterisk en plus de FusionPBX.</t>
+          <t>Formulaire CRUD pbx_connectors dans Réglages &gt; Intégrations, sur le modèle SettingsSmtp.vue.</t>
         </is>
       </c>
       <c r="G75" s="102" t="inlineStr">
@@ -5805,17 +5769,17 @@
       </c>
       <c r="H75" s="100" t="inlineStr">
         <is>
-          <t>½j</t>
+          <t>1j</t>
         </is>
       </c>
       <c r="I75" s="100" t="inlineStr">
         <is>
-          <t>backend/tests/</t>
+          <t>frontend/src/components/settings/SettingsTelephony.vue (nouveau)</t>
         </is>
       </c>
       <c r="J75" s="100" t="inlineStr">
         <is>
-          <t>14.1</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="K75" s="100" t="n"/>
@@ -5825,61 +5789,171 @@
     <row r="76">
       <c r="A76" s="98" t="inlineStr">
         <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="B76" s="99" t="inlineStr">
+        <is>
+          <t>Phase 14</t>
+        </is>
+      </c>
+      <c r="C76" s="100" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D76" s="101" t="inlineStr">
+        <is>
+          <t>🔵 Normale</t>
+        </is>
+      </c>
+      <c r="E76" s="100" t="inlineStr">
+        <is>
+          <t>AMIAdapter (Asterisk) — ajouté au même process connecteur</t>
+        </is>
+      </c>
+      <c r="F76" s="100" t="inlineStr">
+        <is>
+          <t>Implémente PBXAdapter, orchestré par le même Core Connector que l'ESLAdapter (pas un second déploiement) : Dial/Hangup/QueueMember normalisés vers le même format standard.</t>
+        </is>
+      </c>
+      <c r="G76" s="102" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="H76" s="100" t="inlineStr">
+        <is>
+          <t>2j</t>
+        </is>
+      </c>
+      <c r="I76" s="100" t="inlineStr">
+        <is>
+          <t>telephony-connector/adapters/ami.py (nouveau)</t>
+        </is>
+      </c>
+      <c r="J76" s="100" t="inlineStr">
+        <is>
+          <t>12.2, 12.4</t>
+        </is>
+      </c>
+      <c r="K76" s="100" t="n"/>
+      <c r="L76" s="100" t="n"/>
+      <c r="M76" s="100" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="98" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="B77" s="99" t="inlineStr">
+        <is>
+          <t>Phase 14</t>
+        </is>
+      </c>
+      <c r="C77" s="100" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="D77" s="101" t="inlineStr">
+        <is>
+          <t>🔵 Normale</t>
+        </is>
+      </c>
+      <c r="E77" s="100" t="inlineStr">
+        <is>
+          <t>Validation architecture Adapter (non-régression ESL)</t>
+        </is>
+      </c>
+      <c r="F77" s="100" t="inlineStr">
+        <is>
+          <t>Vérifier qu'aucun changement API/frontend n'est requis pour supporter Asterisk en plus de FusionPBX.</t>
+        </is>
+      </c>
+      <c r="G77" s="102" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="H77" s="100" t="inlineStr">
+        <is>
+          <t>½j</t>
+        </is>
+      </c>
+      <c r="I77" s="100" t="inlineStr">
+        <is>
+          <t>backend/tests/</t>
+        </is>
+      </c>
+      <c r="J77" s="100" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="K77" s="100" t="n"/>
+      <c r="L77" s="100" t="n"/>
+      <c r="M77" s="100" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="98" t="inlineStr">
+        <is>
           <t>DOC-TEL-1</t>
         </is>
       </c>
-      <c r="B76" s="103" t="inlineStr">
+      <c r="B78" s="103" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C76" s="100" t="inlineStr">
+      <c r="C78" s="100" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="D76" s="104" t="inlineStr">
+      <c r="D78" s="104" t="inlineStr">
         <is>
           <t>🟢 Normale</t>
         </is>
       </c>
-      <c r="E76" s="105" t="inlineStr">
+      <c r="E78" s="105" t="inlineStr">
         <is>
           <t>Rédiger le plan d'intégration Module Téléphonie</t>
         </is>
       </c>
-      <c r="F76" s="105" t="inlineStr">
+      <c r="F78" s="105" t="inlineStr">
         <is>
           <t>Analyse de l'existant (table dormante, flag cosmétique), décisions d'architecture (polling vs WebSocket, String vs enum), phasage détaillé.</t>
         </is>
       </c>
-      <c r="G76" s="106" t="inlineStr">
+      <c r="G78" s="106" t="inlineStr">
         <is>
           <t>Complété</t>
         </is>
       </c>
-      <c r="H76" s="105" t="inlineStr">
+      <c r="H78" s="105" t="inlineStr">
         <is>
           <t>½j</t>
         </is>
       </c>
-      <c r="I76" s="105" t="inlineStr">
+      <c r="I78" s="105" t="inlineStr">
         <is>
           <t>TELEPHONIE_INTEGRATION_PLAN.md (nouveau) · docs/cdc/CDC-Module-Telephonie.md (nouveau)</t>
         </is>
       </c>
-      <c r="J76" s="105" t="n"/>
-      <c r="K76" s="105" t="inlineStr">
+      <c r="J78" s="105" t="n"/>
+      <c r="K78" s="105" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="L76" s="105" t="inlineStr">
+      <c r="L78" s="105" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="M76" s="105" t="n"/>
+      <c r="M78" s="105" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:M28"/>
@@ -5905,7 +5979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="51" min="1" max="1"/>
@@ -6742,6 +6816,33 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>12.10-12.11</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Deux bugs de production corriges (deadlock connecteur, routage WebSocket Nginx) suite au raccordement a un FusionPBX reel</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>A faire</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
docs: documente les Phases 13/14 (Supervision, webhook CDR, Rapports) et ajoute TELEPHONY_CDR_TRACE
README v1.8.0, PROJECT_STRUCTURE, TELEPHONIE_INTEGRATION_PLAN (nouvelle
section 8.6 detaillant les six correctifs successifs du webhook CDR,
chacun valide contre du trafic FusionPBX reel) et DATABASE_SCHEMA (colonnes
agent_status, authorized_ip, cdr_webhook_token/_hash) mis a jour pour
refleter l'etat reellement livre. Renumerotation Phase 14 (webhook CDR,
faite) / Phase 15 (Asterisk AMI, non demarree) pour rester coherent avec le
phasage original.

Ajoute TELEPHONY_CDR_TRACE a backend/.env.example. Suivi des taches
complete (13.1-14.4) dans docs/suivi_taches_permatel.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/suivi_taches_permatel.xlsx
+++ b/docs/suivi_taches_permatel.xlsx
@@ -1832,7 +1832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M78"/>
+  <dimension ref="A1:M84"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="51" min="1" max="1"/>
@@ -5438,74 +5438,74 @@
       </c>
     </row>
     <row r="69" ht="37.5" customHeight="1" s="52">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="51" t="inlineStr">
         <is>
           <t>12.10</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="51" t="inlineStr">
         <is>
           <t>Phase 12</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="51" t="inlineStr">
         <is>
           <t>Connecteur</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="51" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" s="51" t="inlineStr">
         <is>
           <t>Fix deadlock reconnexion concurrente (ESLAdapter)</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="51" t="inlineStr">
         <is>
           <t>Complete le 2026-07-28 : force_reconnect()/stop() ne touchent plus _esl directement (course avec run() sur ESLProtocol.stop() sans timeout, bloquait le connecteur apres Sync). _hard_disconnect() ferme la socket directement, seule la greenlet run() y touche. 5 tests de regression.</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G69" s="51" t="inlineStr">
         <is>
           <t>Complété</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="51" t="inlineStr">
         <is>
           <t>12.11</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="51" t="inlineStr">
         <is>
           <t>Phase 12</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="51" t="inlineStr">
         <is>
           <t>Frontend/Nginx</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" s="51" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E70" s="51" t="inlineStr">
         <is>
           <t>Fix routage WebSocket Socket.IO (panneau live bloque Deconnecte)</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="51" t="inlineStr">
         <is>
           <t>Complete le 2026-07-28 : /socket.io par defaut non proxifie par Nginx (tombait dans le fallback SPA). Deplace sous /api/socket.io (same-origin) + en-tetes Upgrade/Connection ajoutes a la location /api/. Valide de bout en bout contre une vraie stack Docker (nginx + gunicorn eventlet), pas seulement en test unitaire.</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G70" s="51" t="inlineStr">
         <is>
           <t>Complété</t>
         </is>
@@ -5954,6 +5954,318 @@
         </is>
       </c>
       <c r="M78" s="105" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Phase 13</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Relocalisation config Téléphonie sous Intégrations</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Config déplacée de l'onglet Paramètres autonome vers un panneau "Configurer" inline sous Paramètres &gt; Intégrations. Bouton actif dès que channel_telephonie est activé, indépendamment d'un connecteur déjà configuré (tenant_features.py : integrations.telephony = ch['telephonie'] seul).</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>SettingsIntegrations.vue, SettingsView.vue, tenant_features.py</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Phase 13</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Frontend/Backend</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Supervision &gt; Téléphonie (KPIs, appels en cours, files, grille agents)</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Nouvel onglet Supervision, visible ssi canal actif ET connecteur configuré. Grille d'état des agents adossée à une donnée réelle : capture du header FreeSWITCH CC-Agent-Status (mod_callcenter, jusque-là ignoré), normalisé par GET /telephony/agents/status en présence disponible/pause/hors-ligne (défaut hors-ligne si inconnu — jamais fabriqué). Charge = appels traités relatifs au plus sollicité, pas un taux d'occupation.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>SupervisionTelephony.vue, SupervisionView.vue, telephony.py (agents_status), migration 2f54e418e600</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Phase 14</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Webhook CDR (POST /telephony/cdr/ingest/&lt;token&gt;)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Canal d'ingestion complémentaire à l'ESL live, alimenté directement par FusionPBX (mod_json_cdr) à la fin de chaque appel. Jeton PAR CONNECTEUR (généré à la création, régénérable, stocké hashé+chiffré, réaffichable via "Copier le token"), restriction IP optionnelle (authorized_ip). Un CDR produit jusqu'à 3 TelephonyEvent rétrodatés (ringing/answered/terminal), compatible sans modification avec les routes KPI existantes.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>telephony.py (cdr_ingest), pbx.py, migration 9c8b7a6f5e4d, SettingsTelephony.vue</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Phase 14</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Frontend/Backend</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Rapports &gt; Téléphonie (historique + export CSV + enregistrements + export ZIP)</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Nouvel onglet Rapports, visible ssi canal actif. Historique des appels paginé/filtrable avec export CSV (GET /telephony/calls, /calls/export). Section Enregistrements avec écoute/téléchargement (proxy backend, uniquement si recording_url est une URL http(s) exploitable) et export groupé en ZIP (sélection ou filtres, _indisponibles.txt listant les fichiers exclus).</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>ReportCdr.vue, ReportView.vue, telephony.py (calls/recordings routes), telephonyService.js</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>14.3</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Phase 14</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Critique</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Six correctifs successifs du parsing webhook CDR (validés contre trafic FusionPBX réel)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Chaque round découvert et corrigé contre du vrai trafic de production (pas en local) : (1) get_json() sans force=True ; (2) corps réellement x-www-form-urlencoded (cdr=&lt;json&gt;), pas JSON brut ; (3) '&amp;'/'=' littéraux tronquaient la valeur via le parseur form de Werkzeug — remplacé par extraction directe sur le corps brut ; (4) préservation du '+' des numéros E.164 (unquote avant unquote_plus) ; (5) caractères de contrôle bruts (strict=False) ; (6) root cause finale : FusionPBX interpole des en-têtes SIP bruts sans échapper les guillemets internes — _repair_unescaped_quotes() en dernier recours. Voir TELEPHONIE_INTEGRATION_PLAN.md §8.6 pour le détail complet. 21 tests dédiés.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>telephony.py (cdr_ingest, _repair_unescaped_quotes), test_telephony.py</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>14.4</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Phase 14</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Basse</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Trace diagnostique webhook CDR (TELEPHONY_CDR_TRACE)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Activable via TELEPHONY_CDR_TRACE=true (désactivé par défaut). Journalise l'inventaire complet des variables reçues + écrit le payload intégral dans /tmp/cdr_trace_last.json, pour confirmer quelles variables un PBX réel envoie effectivement (cc_queue/cc_agent, exposition des enregistrements) avant d'exploiter de nouveaux champs.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>telephony.py (_trace_cdr_payload), config.py, .env.example</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M28"/>
@@ -5979,7 +6291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="51" min="1" max="1"/>
@@ -6817,29 +7129,61 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="51" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="51" t="inlineStr">
         <is>
           <t>12.10-12.11</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="51" t="inlineStr">
         <is>
           <t>Deux bugs de production corriges (deadlock connecteur, routage WebSocket Nginx) suite au raccordement a un FusionPBX reel</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="51" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="51" t="inlineStr">
         <is>
           <t>Complété</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>13.1-14.4</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Phase 13/14 : config relocalisée sous Intégrations, Supervision temps réel (grille agents CC-Agent-Status), webhook CDR FusionPBX (mod_json_cdr, jeton par connecteur), Rapports &gt; Téléphonie (historique/export CSV/enregistrements/export ZIP). Six correctifs de parsing CDR validés contre trafic réel.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>236 tests backend au total</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: met a jour le registre des taches (correctifs post-audit + Mon Profil)
Ajoute au suivi les 5 elements livres depuis l'audit du 14/08 (commit
3ead38d), non encore traces :
- 4.7 : fix footer masquant les tiroirs d'edition (Orders/Anomalies)
- 5.5 : fix VITE_INACTIVITY_TIMEOUT_MINUTES non propage au build Docker
- 13.3 : fix affichage agent deduit (appels sortants directs)
- 16.4 : colonnes Derniere modification/Cloture le (Commandes/Anomalies)
- 17.1 (nouvelle Phase 17) : vue Mon Profil self-service

Tableau de bord : compteurs Phase 4/5/13/16 mis a jour, nouvelle ligne
Phase 17 inseree. Changelog complete en consequence.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/suivi_taches_permatel.xlsx
+++ b/docs/suivi_taches_permatel.xlsx
@@ -1234,7 +1234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="51" min="1" max="1"/>
@@ -1256,7 +1256,7 @@
     <row r="2" ht="19.5" customHeight="1" s="52">
       <c r="A2" s="54" t="inlineStr">
         <is>
-          <t>Plan d'action · Audit du 2026-05-10 · Dernière mise à jour : 2026-08-14 (exécution à distance ESL + Rapports enrichis ; audit de conformité des statuts)</t>
+          <t>Plan d'action · Audit du 2026-05-10 · Dernière mise à jour : 2026-08-14 (correctifs UI post-audit + colonnes rapport + vue Mon Profil)</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="D12" s="80" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E12" s="80">
         <f>COUNTIFS(Tâches!B4:B200,"Phase 4",Tâches!G4:G200,"Complété")</f>
@@ -1488,7 +1488,7 @@
         </is>
       </c>
       <c r="D13" s="80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" s="80">
         <f>COUNTIFS(Tâches!B4:B200,"Phase 5",Tâches!G4:G200,"Complété")</f>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="D23" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" s="80">
         <f>COUNTIFS(Tâches!B4:B200,"Phase 13",Tâches!G4:G200,"Complété")</f>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="D26" s="51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E26" s="51">
         <f>COUNTIFS(Tâches!B4:B200,"Phase 16",Tâches!G4:G200,"Complété")</f>
@@ -1837,34 +1837,62 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="63" t="inlineStr">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Phase 17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PHASE 17 — Profil utilisateur (self-service)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>~0.5j</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <f>COUNTIFS(Tâches!B4:B200,"Phase 17",Tâches!G4:G200,"Complété")</f>
+        <v/>
+      </c>
+      <c r="F27">
+        <f>IFERROR(E27/D27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="63" t="inlineStr">
         <is>
           <t>LÉGENDE — STATUTS</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="73" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="73" t="inlineStr">
         <is>
           <t>À faire</t>
         </is>
       </c>
-      <c r="B28" s="74" t="inlineStr">
+      <c r="B29" s="74" t="inlineStr">
         <is>
           <t>En cours</t>
         </is>
       </c>
-      <c r="C28" s="75" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="D28" s="76" t="inlineStr">
+      <c r="C29" s="75" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="D29" s="76" t="inlineStr">
         <is>
           <t>Bloqué</t>
         </is>
       </c>
-      <c r="E28" s="77" t="inlineStr">
+      <c r="E29" s="77" t="inlineStr">
         <is>
           <t>Abandonné</t>
         </is>
@@ -1888,7 +1916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="51" min="1" max="1"/>
@@ -6863,6 +6891,271 @@
         </is>
       </c>
       <c r="L92" s="51" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>🟢 Normale</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Fix : footer applicatif masquait les boutons des tiroirs d'édition</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Les overlays EditCommandeDrawer.vue/EditAnomalieDrawer.vue fixaient bottom:0, ignorant la hauteur du &lt;v-footer app&gt; (z-index Vuetify élevé) — la barre ENREGISTRER/ANNULER passait sous le footer. Réserve désormais --v-layout-bottom, symétrique à --v-layout-top déjà utilisé pour l'app-bar.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>frontend/src/components/workspace/EditCommandeDrawer.vue, EditAnomalieDrawer.vue</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Déploiement</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>🟡 Haute</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Fix déploiement : VITE_INACTIVITY_TIMEOUT_MINUTES jamais propagé au build Docker</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Le Dockerfile frontend n'exposait pas VITE_INACTIVITY_TIMEOUT_MINUTES comme ARG et docker-compose.yml ne le passait pas au build — le frontend se rabattait toujours sur son défaut JS (30 min) même quand SESSION_INACTIVITY_TIMEOUT_MINUTES était personnalisé côté backend, déconnectant l'agent côté UI alors que sa session serveur restait valide. Le build frontend dérive désormais VITE_INACTIVITY_TIMEOUT_MINUTES directement de SESSION_INACTIVITY_TIMEOUT_MINUTES (même variable, pas de VITE_* séparée) — impossible de les faire diverger en Docker.</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>frontend/Dockerfile, docker-compose.yml, .env.example, README.md</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Phase 13</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>🟢 Normale</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Fix affichage : agent déduit masqué sur les appels sortants directs</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Le backend déduit déjà l'agent d'un appel sortant hors file (matching caller/callee contre _live_station_agent_lookup) mais ne backfille jamais agent_login, seulement agent_uuid/agent_name. Le tableau « Appels en cours » gatait la cellule Agent sur c.agent_login → toujours « — » malgré une inférence réussie. Corrigé pour s'afficher dès que agent_name OU agent_login est présent, avec un indice visuel (avatar en pointillés + « (déduit) ») quand agent_inferred est vrai.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>frontend/src/components/supervision/SupervisionTelephony.vue</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Limite connue : ne résout que les postes ayant déjà été vus en file au moins une fois (CALLCENTER_AGENT_STATE_CHANGE). Un agent n'ayant jamais rejoint de file reste non résolu — nécessiterait un repli statique sur User.station_extension, non fait à ce stade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>16.4</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Phase 16</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Backend/Frontend</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>🟢 Normale</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Colonnes « Dernière modification »/« Clôturé le » (Commandes/Anomalies)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Ajout de deux colonnes après « Créée le » dans OrdersView.vue/AnomaliesView.vue, chacune précisant l'utilisateur PERMATEL concerné. closed_by_nom ajouté à la sérialisation (manquait, contrairement à created_by_nom/updated_by_nom déjà présents) ; on_status_change() pose désormais closed_by_id en même temps que closed_at (jamais fait jusqu'ici).</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>app/routes/demandes.py, app/services/sla.py, OrdersView.vue, AnomaliesView.vue</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>17.1</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Phase 17</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Backend/Frontend</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>🟢 Normale</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Vue « Mon Profil » — auto-édition identité/mot de passe/avatar</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Nouvel espace self-service (nom, prénom, mot de passe, avatar), accessible via une entrée en fin de menu latéral. Nouvel endpoint PATCH /api/users/me (jwt_required seul, sans role_required, limité à nom/prénom/avatar) — contrairement à PUT /users/&lt;id&gt; qui est ADMIN-only et bloque même un admin s'éditant lui-même. Le changement de mot de passe réutilise l'endpoint self-service déjà existant PATCH /users/&lt;id&gt;/password.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>app/routes/users.py, MonProfilView.vue, Menu2.vue, router/index.js, userService.js, store/auth.js</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
@@ -6892,7 +7185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="51" min="1" max="1"/>
@@ -8556,6 +8849,166 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Fix footer masquant les tiroirs d'édition</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>bottom:0 -&gt; var(--v-layout-bottom, 34px) sur .ecd-overlay/.ead-overlay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Fix VITE_INACTIVITY_TIMEOUT_MINUTES non propagé au build Docker</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Build arg frontend dérivé de SESSION_INACTIVITY_TIMEOUT_MINUTES (backend), plus de variable VITE_ séparée à synchroniser à la main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Fix affichage agent déduit (appels sortants directs)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Gate frontend corrigé (agent_name/agent_login au lieu de agent_login seul) + indice visuel « déduit ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>16.4</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Colonnes Dernière modification/Clôturé le (Commandes/Anomalies)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>closed_by_nom ajouté à la sérialisation ; closed_by_id posé par on_status_change().</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>17.1</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Nouvelle vue Mon Profil (self-service)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>PATCH /api/users/me (jwt_required, sans role ADMIN) pour nom/prénom/avatar ; mot de passe via l'endpoint self-service existant.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: documente la baseline de couverture de tests (5.4)
pytest --cov=app -> 64% global (7735 stmts, 2786 manquants, 398 tests).
Baseline formelle consignee par module dans le suivi des taches. 5.4
passe a 'En cours' : l'objectif 80%+ est deliberement reporte a un
chantier dedie futur (portee trop large pour cette passe, decide avec
l'utilisateur) plutot que d'etre marque Complete sans l'atteindre.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/suivi_taches_permatel.xlsx
+++ b/docs/suivi_taches_permatel.xlsx
@@ -1837,29 +1837,29 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="51" t="inlineStr">
         <is>
           <t>Phase 17</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="51" t="inlineStr">
         <is>
           <t>PHASE 17 — Profil utilisateur (self-service)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="51" t="inlineStr">
         <is>
           <t>~0.5j</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="51">
         <f>COUNTIFS(Tâches!B4:B200,"Phase 17",Tâches!G4:G200,"Complété")</f>
         <v/>
       </c>
-      <c r="F27">
+      <c r="F27" s="51">
         <f>IFERROR(E27/D27,0)</f>
         <v/>
       </c>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G28" s="102" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>En cours</t>
         </is>
       </c>
       <c r="H28" s="100" t="inlineStr">
@@ -3399,7 +3399,7 @@
       <c r="L28" s="100" t="n"/>
       <c r="M28" s="100" t="inlineStr">
         <is>
-          <t>[Audit 14/08] 394 tests backend / 76 connecteur existent (bien au-delà du périmètre initial) mais aucun rapport de couverture formel (pytest --cov) ni test de migration sous Docker Postgres n'a été tracé — objectif implicitement dépassé en volume, non confirmé en % de couverture.</t>
+          <t>Baseline formelle mesuree le 14/08 : pytest --cov=app -&gt; 64% global (7735 stmts, 2786 miss), 398 tests. Points forts (&gt;=95%) : models/ quasi tous, routes/telephony.py 87%, routes/auth.py 85%. Points faibles notables : services/reencrypt.py 0%, routes/settings.py 19%, routes/prestataires.py 20%, scripts/seed_prestataires.py 11%, utils/crypto.py 54%, utils/login_throttle.py 59%, services/sla.py 51%, routes/demandes.py 62%. Objectif 80%+ delibrement reporte a un chantier dedie futur (scope trop large pour cette passe) — decision actee avec l'utilisateur le 14/08.</t>
         </is>
       </c>
     </row>
@@ -6897,265 +6897,265 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="51" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="51" t="inlineStr">
         <is>
           <t>Phase 4</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="51" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D93" s="51" t="inlineStr">
         <is>
           <t>🟢 Normale</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E93" s="51" t="inlineStr">
         <is>
           <t>Fix : footer applicatif masquait les boutons des tiroirs d'édition</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="F93" s="51" t="inlineStr">
         <is>
           <t>Les overlays EditCommandeDrawer.vue/EditAnomalieDrawer.vue fixaient bottom:0, ignorant la hauteur du &lt;v-footer app&gt; (z-index Vuetify élevé) — la barre ENREGISTRER/ANNULER passait sous le footer. Réserve désormais --v-layout-bottom, symétrique à --v-layout-top déjà utilisé pour l'app-bar.</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
+      <c r="G93" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I93" s="51" t="inlineStr">
         <is>
           <t>frontend/src/components/workspace/EditCommandeDrawer.vue, EditAnomalieDrawer.vue</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr">
+      <c r="K93" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr">
+      <c r="L93" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="51" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="51" t="inlineStr">
         <is>
           <t>Phase 5</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C94" s="51" t="inlineStr">
         <is>
           <t>Déploiement</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D94" s="51" t="inlineStr">
         <is>
           <t>🟡 Haute</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="E94" s="51" t="inlineStr">
         <is>
           <t>Fix déploiement : VITE_INACTIVITY_TIMEOUT_MINUTES jamais propagé au build Docker</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr">
+      <c r="F94" s="51" t="inlineStr">
         <is>
           <t>Le Dockerfile frontend n'exposait pas VITE_INACTIVITY_TIMEOUT_MINUTES comme ARG et docker-compose.yml ne le passait pas au build — le frontend se rabattait toujours sur son défaut JS (30 min) même quand SESSION_INACTIVITY_TIMEOUT_MINUTES était personnalisé côté backend, déconnectant l'agent côté UI alors que sa session serveur restait valide. Le build frontend dérive désormais VITE_INACTIVITY_TIMEOUT_MINUTES directement de SESSION_INACTIVITY_TIMEOUT_MINUTES (même variable, pas de VITE_* séparée) — impossible de les faire diverger en Docker.</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
+      <c r="G94" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I94" s="51" t="inlineStr">
         <is>
           <t>frontend/Dockerfile, docker-compose.yml, .env.example, README.md</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr">
+      <c r="K94" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr">
+      <c r="L94" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="51" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B95" s="51" t="inlineStr">
         <is>
           <t>Phase 13</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C95" s="51" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D95" s="51" t="inlineStr">
         <is>
           <t>🟢 Normale</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
+      <c r="E95" s="51" t="inlineStr">
         <is>
           <t>Fix affichage : agent déduit masqué sur les appels sortants directs</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
+      <c r="F95" s="51" t="inlineStr">
         <is>
           <t>Le backend déduit déjà l'agent d'un appel sortant hors file (matching caller/callee contre _live_station_agent_lookup) mais ne backfille jamais agent_login, seulement agent_uuid/agent_name. Le tableau « Appels en cours » gatait la cellule Agent sur c.agent_login → toujours « — » malgré une inférence réussie. Corrigé pour s'afficher dès que agent_name OU agent_login est présent, avec un indice visuel (avatar en pointillés + « (déduit) ») quand agent_inferred est vrai.</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
+      <c r="G95" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I95" s="51" t="inlineStr">
         <is>
           <t>frontend/src/components/supervision/SupervisionTelephony.vue</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr">
+      <c r="K95" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="L95" t="inlineStr">
+      <c r="L95" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr">
+      <c r="M95" s="51" t="inlineStr">
         <is>
           <t>Limite connue : ne résout que les postes ayant déjà été vus en file au moins une fois (CALLCENTER_AGENT_STATE_CHANGE). Un agent n'ayant jamais rejoint de file reste non résolu — nécessiterait un repli statique sur User.station_extension, non fait à ce stade.</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="51" t="inlineStr">
         <is>
           <t>16.4</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="51" t="inlineStr">
         <is>
           <t>Phase 16</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="51" t="inlineStr">
         <is>
           <t>Backend/Frontend</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D96" s="51" t="inlineStr">
         <is>
           <t>🟢 Normale</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="E96" s="51" t="inlineStr">
         <is>
           <t>Colonnes « Dernière modification »/« Clôturé le » (Commandes/Anomalies)</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
+      <c r="F96" s="51" t="inlineStr">
         <is>
           <t>Ajout de deux colonnes après « Créée le » dans OrdersView.vue/AnomaliesView.vue, chacune précisant l'utilisateur PERMATEL concerné. closed_by_nom ajouté à la sérialisation (manquait, contrairement à created_by_nom/updated_by_nom déjà présents) ; on_status_change() pose désormais closed_by_id en même temps que closed_at (jamais fait jusqu'ici).</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
+      <c r="G96" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I96" s="51" t="inlineStr">
         <is>
           <t>app/routes/demandes.py, app/services/sla.py, OrdersView.vue, AnomaliesView.vue</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr">
+      <c r="K96" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr">
+      <c r="L96" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="51" t="inlineStr">
         <is>
           <t>17.1</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="51" t="inlineStr">
         <is>
           <t>Phase 17</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="51" t="inlineStr">
         <is>
           <t>Backend/Frontend</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D97" s="51" t="inlineStr">
         <is>
           <t>🟢 Normale</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
+      <c r="E97" s="51" t="inlineStr">
         <is>
           <t>Vue « Mon Profil » — auto-édition identité/mot de passe/avatar</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr">
+      <c r="F97" s="51" t="inlineStr">
         <is>
           <t>Nouvel espace self-service (nom, prénom, mot de passe, avatar), accessible via une entrée en fin de menu latéral. Nouvel endpoint PATCH /api/users/me (jwt_required seul, sans role_required, limité à nom/prénom/avatar) — contrairement à PUT /users/&lt;id&gt; qui est ADMIN-only et bloque même un admin s'éditant lui-même. Le changement de mot de passe réutilise l'endpoint self-service déjà existant PATCH /users/&lt;id&gt;/password.</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
+      <c r="G97" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="I97" s="51" t="inlineStr">
         <is>
           <t>app/routes/users.py, MonProfilView.vue, Menu2.vue, router/index.js, userService.js, store/auth.js</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
+      <c r="K97" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="L97" t="inlineStr">
+      <c r="L97" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
@@ -7185,7 +7185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="51" min="1" max="1"/>
@@ -8850,162 +8850,194 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="51" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="51" t="inlineStr">
         <is>
           <t>Fix footer masquant les tiroirs d'édition</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="51" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
+      <c r="E64" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F64" s="51" t="inlineStr">
         <is>
           <t>bottom:0 -&gt; var(--v-layout-bottom, 34px) sur .ecd-overlay/.ead-overlay.</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="51" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="51" t="inlineStr">
         <is>
           <t>Fix VITE_INACTIVITY_TIMEOUT_MINUTES non propagé au build Docker</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="51" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
+      <c r="E65" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F65" s="51" t="inlineStr">
         <is>
           <t>Build arg frontend dérivé de SESSION_INACTIVITY_TIMEOUT_MINUTES (backend), plus de variable VITE_ séparée à synchroniser à la main.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="51" t="inlineStr">
         <is>
           <t>13.3</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="51" t="inlineStr">
         <is>
           <t>Fix affichage agent déduit (appels sortants directs)</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="51" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
+      <c r="E66" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F66" s="51" t="inlineStr">
         <is>
           <t>Gate frontend corrigé (agent_name/agent_login au lieu de agent_login seul) + indice visuel « déduit ».</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="51" t="inlineStr">
         <is>
           <t>16.4</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="51" t="inlineStr">
         <is>
           <t>Colonnes Dernière modification/Clôturé le (Commandes/Anomalies)</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="51" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
+      <c r="E67" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F67" s="51" t="inlineStr">
         <is>
           <t>closed_by_nom ajouté à la sérialisation ; closed_by_id posé par on_status_change().</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="51" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="51" t="inlineStr">
         <is>
           <t>17.1</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="51" t="inlineStr">
         <is>
           <t>Nouvelle vue Mon Profil (self-service)</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="51" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Complété</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
+      <c r="E68" s="51" t="inlineStr">
+        <is>
+          <t>Complété</t>
+        </is>
+      </c>
+      <c r="F68" s="51" t="inlineStr">
         <is>
           <t>PATCH /api/users/me (jwt_required, sans role ADMIN) pour nom/prénom/avatar ; mot de passe via l'endpoint self-service existant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Baseline formelle de couverture de tests (pytest --cov)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>64% global mesure et documente par module ; objectif 80%+ reporte a un chantier dedie futur (decision utilisateur).</t>
         </is>
       </c>
     </row>

</xml_diff>